<commit_message>
Add Tile and fix blueprint
</commit_message>
<xml_diff>
--- a/ARQVJ2026-main/Assets/StreamingAssets/Blueprints/Blueprints.xlsx
+++ b/ARQVJ2026-main/Assets/StreamingAssets/Blueprints/Blueprints.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Animals" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Tile Types" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,48 +11,54 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="16">
   <si>
     <t>IDS</t>
   </si>
   <si>
-    <t>Life</t>
+    <t>Is Structure</t>
   </si>
   <si>
-    <t>Food</t>
+    <t>Is Walkable</t>
   </si>
   <si>
-    <t>Name</t>
+    <t>Is Animal Habitat</t>
   </si>
   <si>
-    <t>Monkey</t>
+    <t>Can Spawn Humans</t>
   </si>
   <si>
-    <t>100,200</t>
+    <t>Can Dispawn Humans</t>
   </si>
   <si>
-    <t>20</t>
+    <t>Is Default</t>
   </si>
   <si>
-    <t>Pepe</t>
+    <t>Road</t>
   </si>
   <si>
-    <t>Snake</t>
+    <t>FALSE</t>
   </si>
   <si>
-    <t>3</t>
+    <t>TRUE</t>
   </si>
   <si>
-    <t>Jose</t>
+    <t>Jail walls</t>
   </si>
   <si>
-    <t>RecontraBird</t>
+    <t>Jail habitat</t>
   </si>
   <si>
-    <t>14</t>
+    <t>Power Suply</t>
   </si>
   <si>
-    <t>Piolin!</t>
+    <t>Humans entry</t>
+  </si>
+  <si>
+    <t>Humans exit</t>
+  </si>
+  <si>
+    <t>Grass</t>
   </si>
 </sst>
 </file>
@@ -310,6 +316,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="12.38"/>
+    <col customWidth="1" min="2" max="3" width="9.5"/>
+    <col customWidth="1" min="4" max="4" width="13.63"/>
+    <col customWidth="1" min="5" max="5" width="16.25"/>
+    <col customWidth="1" min="6" max="6" width="17.63"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -324,9 +337,15 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
@@ -349,20 +368,26 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
@@ -385,20 +410,26 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
+      <c r="D3" s="1" t="s">
+        <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>9</v>
+      <c r="E3" s="1" t="s">
+        <v>8</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>10</v>
+      <c r="F3" s="1" t="s">
+        <v>8</v>
       </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
@@ -424,17 +455,23 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="E4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -457,20 +494,26 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+      <c r="E5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -492,13 +535,27 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -520,13 +577,27 @@
       <c r="Z6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -548,13 +619,27 @@
       <c r="Z7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+      <c r="A8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>

</xml_diff>

<commit_message>
Update DayStep and DayCycle
</commit_message>
<xml_diff>
--- a/ARQVJ2026-main/Assets/StreamingAssets/Blueprints/Blueprints.xlsx
+++ b/ARQVJ2026-main/Assets/StreamingAssets/Blueprints/Blueprints.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Tile Types" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Day Night Cycle" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="24">
   <si>
     <t>IDS</t>
   </si>
@@ -60,6 +61,30 @@
   <si>
     <t>Grass</t>
   </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>Morning</t>
+  </si>
+  <si>
+    <t>MidDay</t>
+  </si>
+  <si>
+    <t>Afternoon</t>
+  </si>
+  <si>
+    <t>Evening</t>
+  </si>
+  <si>
+    <t>Sunrise</t>
+  </si>
+  <si>
+    <t>Dusk</t>
+  </si>
 </sst>
 </file>
 
@@ -92,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -100,6 +125,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -109,6 +137,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -28439,4 +28471,93 @@
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="3">
+        <v>60.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="3">
+        <v>60.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="3">
+        <v>60.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="3">
+        <v>60.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="3">
+        <v>60.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="3">
+        <v>60.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Now you can spawn group of entities
</commit_message>
<xml_diff>
--- a/ARQVJ2026-main/Assets/StreamingAssets/Blueprints/Blueprints.xlsx
+++ b/ARQVJ2026-main/Assets/StreamingAssets/Blueprints/Blueprints.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="61">
   <si>
     <t>IDS</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>Is Default</t>
+  </si>
+  <si>
+    <t>Is Unique</t>
   </si>
   <si>
     <t>Road</t>
@@ -511,7 +514,9 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2"/>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
@@ -533,27 +538,29 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
@@ -575,27 +582,29 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
@@ -617,27 +626,29 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="F4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -659,27 +670,29 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
@@ -701,27 +714,29 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>8</v>
+      <c r="E6" s="1" t="s">
+        <v>10</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>8</v>
+      <c r="G6" s="1" t="s">
+        <v>9</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>8</v>
+      <c r="H6" s="1" t="s">
+        <v>10</v>
       </c>
-      <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
@@ -743,27 +758,29 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="E7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>8</v>
+      <c r="H7" s="1" t="s">
+        <v>10</v>
       </c>
-      <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
@@ -785,27 +802,29 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
@@ -28622,87 +28641,87 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="C8" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -28727,32 +28746,32 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -28777,21 +28796,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -28815,54 +28834,54 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -28882,18 +28901,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C2" s="3">
         <v>60.0</v>
@@ -28901,10 +28920,10 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C3" s="3">
         <v>60.0</v>
@@ -28912,10 +28931,10 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C4" s="3">
         <v>60.0</v>
@@ -28923,10 +28942,10 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C5" s="3">
         <v>60.0</v>
@@ -28934,10 +28953,10 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C6" s="3">
         <v>60.0</v>
@@ -28945,10 +28964,10 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C7" s="3">
         <v>60.0</v>
@@ -28974,18 +28993,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C2" s="3">
         <v>1.0</v>
@@ -28993,10 +29012,10 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C3" s="3">
         <v>1.0</v>
@@ -29004,10 +29023,10 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C4" s="3">
         <v>1.0</v>
@@ -29015,10 +29034,10 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C5" s="3">
         <v>1.0</v>

</xml_diff>